<commit_message>
added multi agent recommender system
</commit_message>
<xml_diff>
--- a/apps_nicolo/LogicCircuits_4s_6r_NLP_MAK_REINFORCE/LogicCircuits_4s_6r_NLP_MAK_REINFORCE_SIL.xlsx
+++ b/apps_nicolo/LogicCircuits_4s_6r_NLP_MAK_REINFORCE/LogicCircuits_4s_6r_NLP_MAK_REINFORCE_SIL.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data'!$A$1:$Z$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data'!$A$1:$Z$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z12"/>
+  <dimension ref="A1:Z13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -1545,8 +1545,96 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2025-12-17 17:04:20</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/logiccircuits-4s-6r-nlp-mak-reinforce-sil/c0084a95c2f749c393001373b8581361</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H13" t="n">
+        <v>300</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>(6, 5, 4, 1280)</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>5</v>
+      </c>
+      <c r="K13" t="n">
+        <v>1024</v>
+      </c>
+      <c r="L13" t="n">
+        <v>10240</v>
+      </c>
+      <c r="M13" t="n">
+        <v>128</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.001, 'topk_entropy_weight': 1.0, 'remainder_entropy_weight': 1.0, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.0}</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>{'risk': 0.9, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>30</v>
+      </c>
+      <c r="R13" t="n">
+        <v>100</v>
+      </c>
+      <c r="S13" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T13" t="n">
+        <v>1</v>
+      </c>
+      <c r="U13" t="n">
+        <v>16</v>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>{'structure': 2.0, 'continuous': 1.0, 'discrete': 0.0, 'input_influence': 0.0}</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>{'target_entropy_ratio_to_max': np.float64(0.26634712992371384), 'initial_temperature': 1.0, 'rate': 0.0, 'current_temperature': 1.0}</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>{'sil_loss_weight': 1.0, 'sil_use_adaptive_baseline': False, 'sil_baseline_annealing_rate': 0.95}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Z12"/>
+  <autoFilter ref="A1:Z13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>